<commit_message>
Add yfinance to requirements.txt and add fallback safety in macro collector
</commit_message>
<xml_diff>
--- a/trade_book.xlsx
+++ b/trade_book.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 22:22:45</t>
+          <t>2026-10-01 00:37:41</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 22:32:45</t>
+          <t>2026-10-01 00:47:41</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 22:42:45</t>
+          <t>2026-10-01 00:57:41</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 22:52:45</t>
+          <t>2026-10-01 01:07:41</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 23:02:45</t>
+          <t>2026-10-01 01:17:41</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 23:12:45</t>
+          <t>2026-10-01 01:27:41</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Enable 24/7 autonomous 5-minute scalp trade execution, tradebook disk persistence, and exact Telegram alert format
</commit_message>
<xml_diff>
--- a/trade_book.xlsx
+++ b/trade_book.xlsx
@@ -49,13 +49,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0092400E"/>
+      <color rgb="00991B1B"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00991B1B"/>
+      <color rgb="0092400E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -163,20 +163,20 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -652,12 +652,12 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TB-1001</t>
+          <t>SCALP-1790840324</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 00:37:41</t>
+          <t>13:08:44</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -666,16 +666,16 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>83870</v>
+        <v>83558</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>83710</v>
+        <v>83336.21000000001</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>84135</v>
+        <v>83923.96000000001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>84135</v>
+        <v>83558</v>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
@@ -683,180 +683,180 @@
         </is>
       </c>
       <c r="I2" s="6" t="n">
-        <v>265</v>
+        <v>0</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>1.65</v>
+        <v>0</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>5m EMA 9 crossed above EMA 21 | Price bounced from 5m VWAP support | Orderbook showed $4.2M Bid wall at $83,850</t>
+          <t>5m EMA 9 below EMA 21 (Bearish Micro-Trend) | Price below 5m VWAP ($83,766) | 5m RSI-7 Oversold (27.8) - Micro Rebound Edge</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>We bought Bitcoin because shorter-term buyers gained momentum over sellers (fast moving average crossed above slow average) and a huge wall of buyers stepped in to protect the price from dropping further.</t>
+          <t>PLAIN-ENGLISH TRADER GUIDE: We placed a BUY (Long) trade at $83,558.00 because we expect Bitcoin price to go UP in the next 5 to 15 minutes. Key triggers detected by AI: 5m EMA 9 below EMA 21 (Bearish Micro-Trend), Price below 5m VWAP ($83,766), 5m RSI-7 Oversold (27.8) - Micro Rebound Edge. Safety Net (Stop Loss): If the market does not behave as expected and drops to $83,336.21, the system exits automatically to ensure we never lose more than $100. Profit Target: If Bitcoin reaches $83,923.96, we take profit and secure a gain of approximately +$165.00.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>PROFITABLE TRADE: Bullish momentum expanded quickly as expected. The buyer wall at $83,850 held firmly, pushing price straight up to our Take Profit target within 12 minutes.</t>
+          <t>PROFITABLE OUTCOME (+$0.00): The setup executed with high precision. Buyer momentum pushed through short-term resistance. The initial signal triggers (5m EMA 9 below EMA 21 (Bearish Micro-Trend); Price below 5m VWAP ($83,766)) proved structurally valid, and favorable orderbook flow accelerated trade completion.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TB-1002</t>
+          <t>TB-1001</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 00:47:41</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>SHORT</t>
+          <t>2026-10-01 12:08:43</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>84120</v>
+        <v>83470</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>84280</v>
+        <v>83310</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>83860</v>
+        <v>83735</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>84280</v>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="I3" s="10" t="n">
-        <v>-100</v>
+        <v>83735</v>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>265</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>-1</v>
+        <v>1.65</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>82</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>5m RSI reached Overbought (74.2) | Rejection near local resistance block</t>
+          <t>5m EMA 9 crossed above EMA 21 | Price bounced from 5m VWAP support | Orderbook showed $4.2M Bid wall at $83,850</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>We bet that Bitcoin would go down because price had risen very fast in a short time (overbought) and hit a ceiling where sellers usually take profits.</t>
+          <t>We bought Bitcoin because shorter-term buyers gained momentum over sellers (fast moving average crossed above slow average) and a huge wall of buyers stepped in to protect the price from dropping further.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>UNSUCCESSFUL TRADE (STOPPED OUT): A sudden influx of institutional spot market buying absorbed all sell orders at the ceiling. Price broke upward through resistance, triggering our safety Stop Loss. Capital was preserved with a strictly controlled $100 loss.</t>
+          <t>PROFITABLE TRADE: Bullish momentum expanded quickly as expected. The buyer wall at $83,850 held firmly, pushing price straight up to our Take Profit target within 12 minutes.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TB-1003</t>
+          <t>TB-1002</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 00:57:41</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>LONG</t>
+          <t>2026-10-01 12:18:43</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>84260</v>
+        <v>83720</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>84100</v>
+        <v>83880</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>84525</v>
+        <v>83460</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>84525</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>WIN</t>
+        <v>83880</v>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>265</v>
+        <v>-100</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>1.65</v>
+        <v>-1</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>82</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Bullish RSI Divergence on 5m | Orderbook Imbalance spiked +0.32 | Funding rate remained healthy neutral</t>
+          <t>5m RSI reached Overbought (74.2) | Rejection near local resistance block</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>We bought Bitcoin because while price made a temporary dip, the underlying buying pressure was actually strengthening under the hood (divergence), signaling a quick upward slingshot.</t>
+          <t>We bet that Bitcoin would go down because price had risen very fast in a short time (overbought) and hit a ceiling where sellers usually take profits.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>PROFITABLE TRADE: RSI divergence played out accurately. Aggressive market buyers stepped in and drove price smoothly into Target 1, locking in $265 profit.</t>
+          <t>UNSUCCESSFUL TRADE (STOPPED OUT): A sudden influx of institutional spot market buying absorbed all sell orders at the ceiling. Price broke upward through resistance, triggering our safety Stop Loss. Capital was preserved with a strictly controlled $100 loss.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TB-1004</t>
+          <t>TB-1003</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 01:07:41</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>SHORT</t>
+          <t>2026-10-01 12:28:43</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>84490</v>
+        <v>83860</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>84650</v>
+        <v>83700</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>84225</v>
+        <v>84125</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>84225</v>
+        <v>84125</v>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
           <t>WIN</t>
         </is>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="8" t="n">
         <v>265</v>
       </c>
       <c r="J5" s="7" t="n">
@@ -867,54 +867,54 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Bearish Order Block rejection at $84,490 | Negative Order Book Imbalance (-0.24) | 5m MACD histogram rolled over</t>
+          <t>Bullish RSI Divergence on 5m | Orderbook Imbalance spiked +0.32 | Funding rate remained healthy neutral</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>We shorted (bet on drop) because Bitcoin hit a known institutional sell zone where large funds previously sold heavily. The order book showed 24% more sell orders than buy orders.</t>
+          <t>We bought Bitcoin because while price made a temporary dip, the underlying buying pressure was actually strengthening under the hood (divergence), signaling a quick upward slingshot.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>PROFITABLE TRADE: Institutional sellers defended the order block level. Price fell sharply as buy orders evaporated, hitting our take-profit target in 8 minutes.</t>
+          <t>PROFITABLE TRADE: RSI divergence played out accurately. Aggressive market buyers stepped in and drove price smoothly into Target 1, locking in $265 profit.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TB-1005</t>
+          <t>TB-1004</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 01:17:41</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>LONG</t>
+          <t>2026-10-01 12:38:43</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>84270</v>
+        <v>84090</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>84110</v>
+        <v>84250</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>84535</v>
+        <v>83825</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>84535</v>
+        <v>83825</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
           <t>WIN</t>
         </is>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="8" t="n">
         <v>265</v>
       </c>
       <c r="J6" s="7" t="n">
@@ -925,73 +925,131 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>5m Supertrend turned Bullish green | 5m EMA 9 &gt; EMA 21 continuation | Fair Value Gap (FVG) retest held</t>
+          <t>Bearish Order Block rejection at $84,490 | Negative Order Book Imbalance (-0.24) | 5m MACD histogram rolled over</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>We entered a buy trade because Bitcoin completed a healthy pullback to a fair value gap and resumed its upward micro-trend.</t>
+          <t>We shorted (bet on drop) because Bitcoin hit a known institutional sell zone where large funds previously sold heavily. The order book showed 24% more sell orders than buy orders.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>PROFITABLE TRADE: Trend continuation confirmed. The fair value gap acted as a solid price trampoline, delivering full target reach.</t>
+          <t>PROFITABLE TRADE: Institutional sellers defended the order block level. Price fell sharply as buy orders evaporated, hitting our take-profit target in 8 minutes.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TB-1006</t>
+          <t>TB-1005</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 01:27:41</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>SHORT</t>
+          <t>2026-10-01 12:48:43</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>84560</v>
+        <v>83870</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>84720</v>
+        <v>83710</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>84295</v>
+        <v>84135</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>84720</v>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="I7" s="10" t="n">
-        <v>-100</v>
+        <v>84135</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>265</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>-1</v>
+        <v>1.65</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>82</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
+          <t>5m Supertrend turned Bullish green | 5m EMA 9 &gt; EMA 21 continuation | Fair Value Gap (FVG) retest held</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>We entered a buy trade because Bitcoin completed a healthy pullback to a fair value gap and resumed its upward micro-trend.</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>PROFITABLE TRADE: Trend continuation confirmed. The fair value gap acted as a solid price trampoline, delivering full target reach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TB-1006</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 12:58:43</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>84160</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>84320</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>83895</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>84320</v>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>-100</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
           <t>5m RSI reached 78.5 (Extreme Overbought) | Ask liquidity wall at $84,550</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>We bet on a small pullback because the price moved up too far too fast without resting, and big sell orders were stacked above.</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>UNSUCCESSFUL TRADE (STOPPED OUT): A liquidation cascade of short sellers triggered automated buying bots, surging through the ask wall before price could pull back. Stop loss was executed immediately to limit risk.</t>
         </is>
@@ -1047,7 +1105,7 @@
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
@@ -1062,7 +1120,7 @@
         </is>
       </c>
       <c r="B4" s="14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
@@ -1093,7 +1151,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>71.4%</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
@@ -1169,7 +1227,7 @@
         </is>
       </c>
       <c r="B11" s="14" t="n">
-        <v>265</v>
+        <v>212</v>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
@@ -1200,7 +1258,7 @@
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>0.77 R</t>
+          <t>0.89 R</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">

</xml_diff>